<commit_message>
Add 2BA st.4.5m with dedicated insulator display counts
</commit_message>
<xml_diff>
--- a/Newdata.xlsx
+++ b/Newdata.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BaseData" sheetId="1" r:id="R8a63f0c5294745a7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BaseData" sheetId="1" r:id="R5ddaa2b84a8a4f2c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -9437,8 +9437,433 @@
         <x:v>1</x:v>
       </x:c>
     </x:row>
+    <x:row r="466">
+      <x:c r="A466">
+        <x:v>12.2</x:v>
+      </x:c>
+      <x:c r="B466" t="str">
+        <x:v>2BA st.4.5m</x:v>
+      </x:c>
+      <x:c r="C466" t="s">
+        <x:v>83</x:v>
+      </x:c>
+      <x:c r="D466" t="s">
+        <x:v>84</x:v>
+      </x:c>
+      <x:c r="E466">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="467">
+      <x:c r="A467">
+        <x:v>12.2</x:v>
+      </x:c>
+      <x:c r="B467" t="str">
+        <x:v>2BA st.4.5m</x:v>
+      </x:c>
+      <x:c r="C467" t="s">
+        <x:v>173</x:v>
+      </x:c>
+      <x:c r="D467" t="s">
+        <x:v>174</x:v>
+      </x:c>
+      <x:c r="E467">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="468">
+      <x:c r="A468">
+        <x:v>12.2</x:v>
+      </x:c>
+      <x:c r="B468" t="str">
+        <x:v>2BA st.4.5m</x:v>
+      </x:c>
+      <x:c r="C468" t="s">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="D468">
+        <x:v>1010110202</x:v>
+      </x:c>
+      <x:c r="E468">
+        <x:v>4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="469">
+      <x:c r="A469">
+        <x:v>12.2</x:v>
+      </x:c>
+      <x:c r="B469" t="str">
+        <x:v>2BA st.4.5m</x:v>
+      </x:c>
+      <x:c r="C469" t="s">
+        <x:v>87</x:v>
+      </x:c>
+      <x:c r="D469">
+        <x:v>1010130001</x:v>
+      </x:c>
+      <x:c r="E469">
+        <x:v>-2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="470">
+      <x:c r="A470">
+        <x:v>12.2</x:v>
+      </x:c>
+      <x:c r="B470" t="str">
+        <x:v>2BA st.4.5m</x:v>
+      </x:c>
+      <x:c r="C470" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="D470">
+        <x:v>1010180100</x:v>
+      </x:c>
+      <x:c r="E470">
+        <x:v>12</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="471">
+      <x:c r="A471">
+        <x:v>12.2</x:v>
+      </x:c>
+      <x:c r="B471" t="str">
+        <x:v>2BA st.4.5m</x:v>
+      </x:c>
+      <x:c r="C471" t="s">
+        <x:v>199</x:v>
+      </x:c>
+      <x:c r="D471">
+        <x:v>1010180001</x:v>
+      </x:c>
+      <x:c r="E471">
+        <x:v>6</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="472">
+      <x:c r="A472">
+        <x:v>12.2</x:v>
+      </x:c>
+      <x:c r="B472" t="str">
+        <x:v>2BA st.4.5m</x:v>
+      </x:c>
+      <x:c r="C472" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="D472">
+        <x:v>1010180301</x:v>
+      </x:c>
+      <x:c r="E472">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="473">
+      <x:c r="A473">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="B473" t="str">
+        <x:v>2BA st.4.5m</x:v>
+      </x:c>
+      <x:c r="C473" t="s">
+        <x:v>83</x:v>
+      </x:c>
+      <x:c r="D473" t="s">
+        <x:v>84</x:v>
+      </x:c>
+      <x:c r="E473">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="474">
+      <x:c r="A474">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="B474" t="str">
+        <x:v>2BA st.4.5m</x:v>
+      </x:c>
+      <x:c r="C474" t="s">
+        <x:v>173</x:v>
+      </x:c>
+      <x:c r="D474" t="s">
+        <x:v>174</x:v>
+      </x:c>
+      <x:c r="E474">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="475">
+      <x:c r="A475">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="B475" t="str">
+        <x:v>2BA st.4.5m</x:v>
+      </x:c>
+      <x:c r="C475" t="s">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="D475">
+        <x:v>1010110202</x:v>
+      </x:c>
+      <x:c r="E475">
+        <x:v>4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="476">
+      <x:c r="A476">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="B476" t="str">
+        <x:v>2BA st.4.5m</x:v>
+      </x:c>
+      <x:c r="C476" t="s">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="D476">
+        <x:v>1010110207</x:v>
+      </x:c>
+      <x:c r="E476">
+        <x:v>-1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="477">
+      <x:c r="A477">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="B477" t="str">
+        <x:v>2BA st.4.5m</x:v>
+      </x:c>
+      <x:c r="C477" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="D477">
+        <x:v>1010110209</x:v>
+      </x:c>
+      <x:c r="E477">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="478">
+      <x:c r="A478">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="B478" t="str">
+        <x:v>2BA st.4.5m</x:v>
+      </x:c>
+      <x:c r="C478" t="s">
+        <x:v>87</x:v>
+      </x:c>
+      <x:c r="D478">
+        <x:v>1010130001</x:v>
+      </x:c>
+      <x:c r="E478">
+        <x:v>-2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="479">
+      <x:c r="A479">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="B479" t="str">
+        <x:v>2BA st.4.5m</x:v>
+      </x:c>
+      <x:c r="C479" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="D479">
+        <x:v>1010180100</x:v>
+      </x:c>
+      <x:c r="E479">
+        <x:v>12</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="480">
+      <x:c r="A480">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="B480" t="str">
+        <x:v>2BA st.4.5m</x:v>
+      </x:c>
+      <x:c r="C480" t="s">
+        <x:v>199</x:v>
+      </x:c>
+      <x:c r="D480">
+        <x:v>1010180001</x:v>
+      </x:c>
+      <x:c r="E480">
+        <x:v>6</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="481">
+      <x:c r="A481">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="B481" t="str">
+        <x:v>2BA st.4.5m</x:v>
+      </x:c>
+      <x:c r="C481" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="D481">
+        <x:v>1010180301</x:v>
+      </x:c>
+      <x:c r="E481">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="482">
+      <x:c r="A482">
+        <x:v>14.3</x:v>
+      </x:c>
+      <x:c r="B482" t="str">
+        <x:v>2BA st.4.5m</x:v>
+      </x:c>
+      <x:c r="C482" t="s">
+        <x:v>83</x:v>
+      </x:c>
+      <x:c r="D482" t="s">
+        <x:v>84</x:v>
+      </x:c>
+      <x:c r="E482">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="483">
+      <x:c r="A483">
+        <x:v>14.3</x:v>
+      </x:c>
+      <x:c r="B483" t="str">
+        <x:v>2BA st.4.5m</x:v>
+      </x:c>
+      <x:c r="C483" t="s">
+        <x:v>173</x:v>
+      </x:c>
+      <x:c r="D483" t="s">
+        <x:v>174</x:v>
+      </x:c>
+      <x:c r="E483">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="484">
+      <x:c r="A484">
+        <x:v>14.3</x:v>
+      </x:c>
+      <x:c r="B484" t="str">
+        <x:v>2BA st.4.5m</x:v>
+      </x:c>
+      <x:c r="C484" t="s">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="D484">
+        <x:v>1010110202</x:v>
+      </x:c>
+      <x:c r="E484">
+        <x:v>4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="485">
+      <x:c r="A485">
+        <x:v>14.3</x:v>
+      </x:c>
+      <x:c r="B485" t="str">
+        <x:v>2BA st.4.5m</x:v>
+      </x:c>
+      <x:c r="C485" t="s">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="D485">
+        <x:v>1010110207</x:v>
+      </x:c>
+      <x:c r="E485">
+        <x:v>-1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="486">
+      <x:c r="A486">
+        <x:v>14.3</x:v>
+      </x:c>
+      <x:c r="B486" t="str">
+        <x:v>2BA st.4.5m</x:v>
+      </x:c>
+      <x:c r="C486" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="D486">
+        <x:v>1010110209</x:v>
+      </x:c>
+      <x:c r="E486">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="487">
+      <x:c r="A487">
+        <x:v>14.3</x:v>
+      </x:c>
+      <x:c r="B487" t="str">
+        <x:v>2BA st.4.5m</x:v>
+      </x:c>
+      <x:c r="C487" t="s">
+        <x:v>87</x:v>
+      </x:c>
+      <x:c r="D487">
+        <x:v>1010130001</x:v>
+      </x:c>
+      <x:c r="E487">
+        <x:v>-2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="488">
+      <x:c r="A488">
+        <x:v>14.3</x:v>
+      </x:c>
+      <x:c r="B488" t="str">
+        <x:v>2BA st.4.5m</x:v>
+      </x:c>
+      <x:c r="C488" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="D488">
+        <x:v>1010180100</x:v>
+      </x:c>
+      <x:c r="E488">
+        <x:v>12</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="489">
+      <x:c r="A489">
+        <x:v>14.3</x:v>
+      </x:c>
+      <x:c r="B489" t="str">
+        <x:v>2BA st.4.5m</x:v>
+      </x:c>
+      <x:c r="C489" t="s">
+        <x:v>199</x:v>
+      </x:c>
+      <x:c r="D489">
+        <x:v>1010180001</x:v>
+      </x:c>
+      <x:c r="E489">
+        <x:v>6</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="490">
+      <x:c r="A490">
+        <x:v>14.3</x:v>
+      </x:c>
+      <x:c r="B490" t="str">
+        <x:v>2BA st.4.5m</x:v>
+      </x:c>
+      <x:c r="C490" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="D490">
+        <x:v>1010180301</x:v>
+      </x:c>
+      <x:c r="E490">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R046f6652d3fe468a"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rba752e7dd8764772"/>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add SP,DDE.BL st.4.5m with insulator display counts
</commit_message>
<xml_diff>
--- a/Newdata.xlsx
+++ b/Newdata.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BaseData" sheetId="1" r:id="R5ddaa2b84a8a4f2c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BaseData" sheetId="1" r:id="Rb4cf1fa8abbe4733"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -9862,8 +9862,433 @@
         <x:v>1</x:v>
       </x:c>
     </x:row>
+    <x:row r="491">
+      <x:c r="A491">
+        <x:v>12.2</x:v>
+      </x:c>
+      <x:c r="B491" t="str">
+        <x:v>SP,DDE.BL st.4.5m</x:v>
+      </x:c>
+      <x:c r="C491" t="s">
+        <x:v>83</x:v>
+      </x:c>
+      <x:c r="D491" t="s">
+        <x:v>84</x:v>
+      </x:c>
+      <x:c r="E491">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="492">
+      <x:c r="A492">
+        <x:v>12.2</x:v>
+      </x:c>
+      <x:c r="B492" t="str">
+        <x:v>SP,DDE.BL st.4.5m</x:v>
+      </x:c>
+      <x:c r="C492" t="s">
+        <x:v>173</x:v>
+      </x:c>
+      <x:c r="D492" t="s">
+        <x:v>174</x:v>
+      </x:c>
+      <x:c r="E492">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="493">
+      <x:c r="A493">
+        <x:v>12.2</x:v>
+      </x:c>
+      <x:c r="B493" t="str">
+        <x:v>SP,DDE.BL st.4.5m</x:v>
+      </x:c>
+      <x:c r="C493" t="s">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="D493">
+        <x:v>1010110202</x:v>
+      </x:c>
+      <x:c r="E493">
+        <x:v>4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="494">
+      <x:c r="A494">
+        <x:v>12.2</x:v>
+      </x:c>
+      <x:c r="B494" t="str">
+        <x:v>SP,DDE.BL st.4.5m</x:v>
+      </x:c>
+      <x:c r="C494" t="s">
+        <x:v>87</x:v>
+      </x:c>
+      <x:c r="D494">
+        <x:v>1010130001</x:v>
+      </x:c>
+      <x:c r="E494">
+        <x:v>-2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="495">
+      <x:c r="A495">
+        <x:v>12.2</x:v>
+      </x:c>
+      <x:c r="B495" t="str">
+        <x:v>SP,DDE.BL st.4.5m</x:v>
+      </x:c>
+      <x:c r="C495" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="D495">
+        <x:v>1010180100</x:v>
+      </x:c>
+      <x:c r="E495">
+        <x:v>12</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="496">
+      <x:c r="A496">
+        <x:v>12.2</x:v>
+      </x:c>
+      <x:c r="B496" t="str">
+        <x:v>SP,DDE.BL st.4.5m</x:v>
+      </x:c>
+      <x:c r="C496" t="s">
+        <x:v>199</x:v>
+      </x:c>
+      <x:c r="D496">
+        <x:v>1010180001</x:v>
+      </x:c>
+      <x:c r="E496">
+        <x:v>6</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="497">
+      <x:c r="A497">
+        <x:v>12.2</x:v>
+      </x:c>
+      <x:c r="B497" t="str">
+        <x:v>SP,DDE.BL st.4.5m</x:v>
+      </x:c>
+      <x:c r="C497" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="D497">
+        <x:v>1010180301</x:v>
+      </x:c>
+      <x:c r="E497">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="498">
+      <x:c r="A498">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="B498" t="str">
+        <x:v>SP,DDE.BL st.4.5m</x:v>
+      </x:c>
+      <x:c r="C498" t="s">
+        <x:v>83</x:v>
+      </x:c>
+      <x:c r="D498" t="s">
+        <x:v>84</x:v>
+      </x:c>
+      <x:c r="E498">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="499">
+      <x:c r="A499">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="B499" t="str">
+        <x:v>SP,DDE.BL st.4.5m</x:v>
+      </x:c>
+      <x:c r="C499" t="s">
+        <x:v>173</x:v>
+      </x:c>
+      <x:c r="D499" t="s">
+        <x:v>174</x:v>
+      </x:c>
+      <x:c r="E499">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="500">
+      <x:c r="A500">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="B500" t="str">
+        <x:v>SP,DDE.BL st.4.5m</x:v>
+      </x:c>
+      <x:c r="C500" t="s">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="D500">
+        <x:v>1010110202</x:v>
+      </x:c>
+      <x:c r="E500">
+        <x:v>4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="501">
+      <x:c r="A501">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="B501" t="str">
+        <x:v>SP,DDE.BL st.4.5m</x:v>
+      </x:c>
+      <x:c r="C501" t="s">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="D501">
+        <x:v>1010110207</x:v>
+      </x:c>
+      <x:c r="E501">
+        <x:v>-1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="502">
+      <x:c r="A502">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="B502" t="str">
+        <x:v>SP,DDE.BL st.4.5m</x:v>
+      </x:c>
+      <x:c r="C502" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="D502">
+        <x:v>1010110209</x:v>
+      </x:c>
+      <x:c r="E502">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="503">
+      <x:c r="A503">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="B503" t="str">
+        <x:v>SP,DDE.BL st.4.5m</x:v>
+      </x:c>
+      <x:c r="C503" t="s">
+        <x:v>87</x:v>
+      </x:c>
+      <x:c r="D503">
+        <x:v>1010130001</x:v>
+      </x:c>
+      <x:c r="E503">
+        <x:v>-2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="504">
+      <x:c r="A504">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="B504" t="str">
+        <x:v>SP,DDE.BL st.4.5m</x:v>
+      </x:c>
+      <x:c r="C504" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="D504">
+        <x:v>1010180100</x:v>
+      </x:c>
+      <x:c r="E504">
+        <x:v>12</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="505">
+      <x:c r="A505">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="B505" t="str">
+        <x:v>SP,DDE.BL st.4.5m</x:v>
+      </x:c>
+      <x:c r="C505" t="s">
+        <x:v>199</x:v>
+      </x:c>
+      <x:c r="D505">
+        <x:v>1010180001</x:v>
+      </x:c>
+      <x:c r="E505">
+        <x:v>6</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="506">
+      <x:c r="A506">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="B506" t="str">
+        <x:v>SP,DDE.BL st.4.5m</x:v>
+      </x:c>
+      <x:c r="C506" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="D506">
+        <x:v>1010180301</x:v>
+      </x:c>
+      <x:c r="E506">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="507">
+      <x:c r="A507">
+        <x:v>14.3</x:v>
+      </x:c>
+      <x:c r="B507" t="str">
+        <x:v>SP,DDE.BL st.4.5m</x:v>
+      </x:c>
+      <x:c r="C507" t="s">
+        <x:v>83</x:v>
+      </x:c>
+      <x:c r="D507" t="s">
+        <x:v>84</x:v>
+      </x:c>
+      <x:c r="E507">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="508">
+      <x:c r="A508">
+        <x:v>14.3</x:v>
+      </x:c>
+      <x:c r="B508" t="str">
+        <x:v>SP,DDE.BL st.4.5m</x:v>
+      </x:c>
+      <x:c r="C508" t="s">
+        <x:v>173</x:v>
+      </x:c>
+      <x:c r="D508" t="s">
+        <x:v>174</x:v>
+      </x:c>
+      <x:c r="E508">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="509">
+      <x:c r="A509">
+        <x:v>14.3</x:v>
+      </x:c>
+      <x:c r="B509" t="str">
+        <x:v>SP,DDE.BL st.4.5m</x:v>
+      </x:c>
+      <x:c r="C509" t="s">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="D509">
+        <x:v>1010110202</x:v>
+      </x:c>
+      <x:c r="E509">
+        <x:v>4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="510">
+      <x:c r="A510">
+        <x:v>14.3</x:v>
+      </x:c>
+      <x:c r="B510" t="str">
+        <x:v>SP,DDE.BL st.4.5m</x:v>
+      </x:c>
+      <x:c r="C510" t="s">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="D510">
+        <x:v>1010110207</x:v>
+      </x:c>
+      <x:c r="E510">
+        <x:v>-1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="511">
+      <x:c r="A511">
+        <x:v>14.3</x:v>
+      </x:c>
+      <x:c r="B511" t="str">
+        <x:v>SP,DDE.BL st.4.5m</x:v>
+      </x:c>
+      <x:c r="C511" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="D511">
+        <x:v>1010110209</x:v>
+      </x:c>
+      <x:c r="E511">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="512">
+      <x:c r="A512">
+        <x:v>14.3</x:v>
+      </x:c>
+      <x:c r="B512" t="str">
+        <x:v>SP,DDE.BL st.4.5m</x:v>
+      </x:c>
+      <x:c r="C512" t="s">
+        <x:v>87</x:v>
+      </x:c>
+      <x:c r="D512">
+        <x:v>1010130001</x:v>
+      </x:c>
+      <x:c r="E512">
+        <x:v>-2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="513">
+      <x:c r="A513">
+        <x:v>14.3</x:v>
+      </x:c>
+      <x:c r="B513" t="str">
+        <x:v>SP,DDE.BL st.4.5m</x:v>
+      </x:c>
+      <x:c r="C513" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="D513">
+        <x:v>1010180100</x:v>
+      </x:c>
+      <x:c r="E513">
+        <x:v>12</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="514">
+      <x:c r="A514">
+        <x:v>14.3</x:v>
+      </x:c>
+      <x:c r="B514" t="str">
+        <x:v>SP,DDE.BL st.4.5m</x:v>
+      </x:c>
+      <x:c r="C514" t="s">
+        <x:v>199</x:v>
+      </x:c>
+      <x:c r="D514">
+        <x:v>1010180001</x:v>
+      </x:c>
+      <x:c r="E514">
+        <x:v>6</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="515">
+      <x:c r="A515">
+        <x:v>14.3</x:v>
+      </x:c>
+      <x:c r="B515" t="str">
+        <x:v>SP,DDE.BL st.4.5m</x:v>
+      </x:c>
+      <x:c r="C515" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="D515">
+        <x:v>1010180301</x:v>
+      </x:c>
+      <x:c r="E515">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rba752e7dd8764772"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rde17b097dd794a8e"/>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add DP,DDE.BL st.4.5m with insulator display counts
</commit_message>
<xml_diff>
--- a/Newdata.xlsx
+++ b/Newdata.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BaseData" sheetId="1" r:id="Rb4cf1fa8abbe4733"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BaseData" sheetId="1" r:id="R062547b4ece24aa0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -10287,8 +10287,433 @@
         <x:v>1</x:v>
       </x:c>
     </x:row>
+    <x:row r="516">
+      <x:c r="A516">
+        <x:v>12.2</x:v>
+      </x:c>
+      <x:c r="B516" t="str">
+        <x:v>DP,DDE.BL st.4.5m</x:v>
+      </x:c>
+      <x:c r="C516" t="s">
+        <x:v>83</x:v>
+      </x:c>
+      <x:c r="D516" t="s">
+        <x:v>84</x:v>
+      </x:c>
+      <x:c r="E516">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="517">
+      <x:c r="A517">
+        <x:v>12.2</x:v>
+      </x:c>
+      <x:c r="B517" t="str">
+        <x:v>DP,DDE.BL st.4.5m</x:v>
+      </x:c>
+      <x:c r="C517" t="s">
+        <x:v>173</x:v>
+      </x:c>
+      <x:c r="D517" t="s">
+        <x:v>174</x:v>
+      </x:c>
+      <x:c r="E517">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="518">
+      <x:c r="A518">
+        <x:v>12.2</x:v>
+      </x:c>
+      <x:c r="B518" t="str">
+        <x:v>DP,DDE.BL st.4.5m</x:v>
+      </x:c>
+      <x:c r="C518" t="s">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="D518">
+        <x:v>1010110202</x:v>
+      </x:c>
+      <x:c r="E518">
+        <x:v>4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="519">
+      <x:c r="A519">
+        <x:v>12.2</x:v>
+      </x:c>
+      <x:c r="B519" t="str">
+        <x:v>DP,DDE.BL st.4.5m</x:v>
+      </x:c>
+      <x:c r="C519" t="s">
+        <x:v>87</x:v>
+      </x:c>
+      <x:c r="D519">
+        <x:v>1010130001</x:v>
+      </x:c>
+      <x:c r="E519">
+        <x:v>-2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="520">
+      <x:c r="A520">
+        <x:v>12.2</x:v>
+      </x:c>
+      <x:c r="B520" t="str">
+        <x:v>DP,DDE.BL st.4.5m</x:v>
+      </x:c>
+      <x:c r="C520" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="D520">
+        <x:v>1010180100</x:v>
+      </x:c>
+      <x:c r="E520">
+        <x:v>12</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="521">
+      <x:c r="A521">
+        <x:v>12.2</x:v>
+      </x:c>
+      <x:c r="B521" t="str">
+        <x:v>DP,DDE.BL st.4.5m</x:v>
+      </x:c>
+      <x:c r="C521" t="s">
+        <x:v>199</x:v>
+      </x:c>
+      <x:c r="D521">
+        <x:v>1010180001</x:v>
+      </x:c>
+      <x:c r="E521">
+        <x:v>6</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="522">
+      <x:c r="A522">
+        <x:v>12.2</x:v>
+      </x:c>
+      <x:c r="B522" t="str">
+        <x:v>DP,DDE.BL st.4.5m</x:v>
+      </x:c>
+      <x:c r="C522" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="D522">
+        <x:v>1010180301</x:v>
+      </x:c>
+      <x:c r="E522">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="523">
+      <x:c r="A523">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="B523" t="str">
+        <x:v>DP,DDE.BL st.4.5m</x:v>
+      </x:c>
+      <x:c r="C523" t="s">
+        <x:v>83</x:v>
+      </x:c>
+      <x:c r="D523" t="s">
+        <x:v>84</x:v>
+      </x:c>
+      <x:c r="E523">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="524">
+      <x:c r="A524">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="B524" t="str">
+        <x:v>DP,DDE.BL st.4.5m</x:v>
+      </x:c>
+      <x:c r="C524" t="s">
+        <x:v>173</x:v>
+      </x:c>
+      <x:c r="D524" t="s">
+        <x:v>174</x:v>
+      </x:c>
+      <x:c r="E524">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="525">
+      <x:c r="A525">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="B525" t="str">
+        <x:v>DP,DDE.BL st.4.5m</x:v>
+      </x:c>
+      <x:c r="C525" t="s">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="D525">
+        <x:v>1010110202</x:v>
+      </x:c>
+      <x:c r="E525">
+        <x:v>4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="526">
+      <x:c r="A526">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="B526" t="str">
+        <x:v>DP,DDE.BL st.4.5m</x:v>
+      </x:c>
+      <x:c r="C526" t="s">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="D526">
+        <x:v>1010110207</x:v>
+      </x:c>
+      <x:c r="E526">
+        <x:v>-1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="527">
+      <x:c r="A527">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="B527" t="str">
+        <x:v>DP,DDE.BL st.4.5m</x:v>
+      </x:c>
+      <x:c r="C527" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="D527">
+        <x:v>1010110209</x:v>
+      </x:c>
+      <x:c r="E527">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="528">
+      <x:c r="A528">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="B528" t="str">
+        <x:v>DP,DDE.BL st.4.5m</x:v>
+      </x:c>
+      <x:c r="C528" t="s">
+        <x:v>87</x:v>
+      </x:c>
+      <x:c r="D528">
+        <x:v>1010130001</x:v>
+      </x:c>
+      <x:c r="E528">
+        <x:v>-2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="529">
+      <x:c r="A529">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="B529" t="str">
+        <x:v>DP,DDE.BL st.4.5m</x:v>
+      </x:c>
+      <x:c r="C529" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="D529">
+        <x:v>1010180100</x:v>
+      </x:c>
+      <x:c r="E529">
+        <x:v>12</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="530">
+      <x:c r="A530">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="B530" t="str">
+        <x:v>DP,DDE.BL st.4.5m</x:v>
+      </x:c>
+      <x:c r="C530" t="s">
+        <x:v>199</x:v>
+      </x:c>
+      <x:c r="D530">
+        <x:v>1010180001</x:v>
+      </x:c>
+      <x:c r="E530">
+        <x:v>6</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="531">
+      <x:c r="A531">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="B531" t="str">
+        <x:v>DP,DDE.BL st.4.5m</x:v>
+      </x:c>
+      <x:c r="C531" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="D531">
+        <x:v>1010180301</x:v>
+      </x:c>
+      <x:c r="E531">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="532">
+      <x:c r="A532">
+        <x:v>14.3</x:v>
+      </x:c>
+      <x:c r="B532" t="str">
+        <x:v>DP,DDE.BL st.4.5m</x:v>
+      </x:c>
+      <x:c r="C532" t="s">
+        <x:v>83</x:v>
+      </x:c>
+      <x:c r="D532" t="s">
+        <x:v>84</x:v>
+      </x:c>
+      <x:c r="E532">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="533">
+      <x:c r="A533">
+        <x:v>14.3</x:v>
+      </x:c>
+      <x:c r="B533" t="str">
+        <x:v>DP,DDE.BL st.4.5m</x:v>
+      </x:c>
+      <x:c r="C533" t="s">
+        <x:v>173</x:v>
+      </x:c>
+      <x:c r="D533" t="s">
+        <x:v>174</x:v>
+      </x:c>
+      <x:c r="E533">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="534">
+      <x:c r="A534">
+        <x:v>14.3</x:v>
+      </x:c>
+      <x:c r="B534" t="str">
+        <x:v>DP,DDE.BL st.4.5m</x:v>
+      </x:c>
+      <x:c r="C534" t="s">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="D534">
+        <x:v>1010110202</x:v>
+      </x:c>
+      <x:c r="E534">
+        <x:v>4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="535">
+      <x:c r="A535">
+        <x:v>14.3</x:v>
+      </x:c>
+      <x:c r="B535" t="str">
+        <x:v>DP,DDE.BL st.4.5m</x:v>
+      </x:c>
+      <x:c r="C535" t="s">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="D535">
+        <x:v>1010110207</x:v>
+      </x:c>
+      <x:c r="E535">
+        <x:v>-1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="536">
+      <x:c r="A536">
+        <x:v>14.3</x:v>
+      </x:c>
+      <x:c r="B536" t="str">
+        <x:v>DP,DDE.BL st.4.5m</x:v>
+      </x:c>
+      <x:c r="C536" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="D536">
+        <x:v>1010110209</x:v>
+      </x:c>
+      <x:c r="E536">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="537">
+      <x:c r="A537">
+        <x:v>14.3</x:v>
+      </x:c>
+      <x:c r="B537" t="str">
+        <x:v>DP,DDE.BL st.4.5m</x:v>
+      </x:c>
+      <x:c r="C537" t="s">
+        <x:v>87</x:v>
+      </x:c>
+      <x:c r="D537">
+        <x:v>1010130001</x:v>
+      </x:c>
+      <x:c r="E537">
+        <x:v>-2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="538">
+      <x:c r="A538">
+        <x:v>14.3</x:v>
+      </x:c>
+      <x:c r="B538" t="str">
+        <x:v>DP,DDE.BL st.4.5m</x:v>
+      </x:c>
+      <x:c r="C538" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="D538">
+        <x:v>1010180100</x:v>
+      </x:c>
+      <x:c r="E538">
+        <x:v>12</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="539">
+      <x:c r="A539">
+        <x:v>14.3</x:v>
+      </x:c>
+      <x:c r="B539" t="str">
+        <x:v>DP,DDE.BL st.4.5m</x:v>
+      </x:c>
+      <x:c r="C539" t="s">
+        <x:v>199</x:v>
+      </x:c>
+      <x:c r="D539">
+        <x:v>1010180001</x:v>
+      </x:c>
+      <x:c r="E539">
+        <x:v>6</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="540">
+      <x:c r="A540">
+        <x:v>14.3</x:v>
+      </x:c>
+      <x:c r="B540" t="str">
+        <x:v>DP,DDE.BL st.4.5m</x:v>
+      </x:c>
+      <x:c r="C540" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="D540">
+        <x:v>1010180301</x:v>
+      </x:c>
+      <x:c r="E540">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rde17b097dd794a8e"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8761d97a3a1f47c8"/>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add DP,DDE st.4.5m with insulator display counts
</commit_message>
<xml_diff>
--- a/Newdata.xlsx
+++ b/Newdata.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BaseData" sheetId="1" r:id="R062547b4ece24aa0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BaseData" sheetId="1" r:id="Rc3d5d22a7d5d4c94"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -10712,8 +10712,433 @@
         <x:v>1</x:v>
       </x:c>
     </x:row>
+    <x:row r="541">
+      <x:c r="A541">
+        <x:v>12.2</x:v>
+      </x:c>
+      <x:c r="B541" t="str">
+        <x:v>DP,DDE st.4.5m</x:v>
+      </x:c>
+      <x:c r="C541" t="s">
+        <x:v>83</x:v>
+      </x:c>
+      <x:c r="D541" t="s">
+        <x:v>84</x:v>
+      </x:c>
+      <x:c r="E541">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="542">
+      <x:c r="A542">
+        <x:v>12.2</x:v>
+      </x:c>
+      <x:c r="B542" t="str">
+        <x:v>DP,DDE st.4.5m</x:v>
+      </x:c>
+      <x:c r="C542" t="s">
+        <x:v>173</x:v>
+      </x:c>
+      <x:c r="D542" t="s">
+        <x:v>174</x:v>
+      </x:c>
+      <x:c r="E542">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="543">
+      <x:c r="A543">
+        <x:v>12.2</x:v>
+      </x:c>
+      <x:c r="B543" t="str">
+        <x:v>DP,DDE st.4.5m</x:v>
+      </x:c>
+      <x:c r="C543" t="s">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="D543">
+        <x:v>1010110202</x:v>
+      </x:c>
+      <x:c r="E543">
+        <x:v>4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="544">
+      <x:c r="A544">
+        <x:v>12.2</x:v>
+      </x:c>
+      <x:c r="B544" t="str">
+        <x:v>DP,DDE st.4.5m</x:v>
+      </x:c>
+      <x:c r="C544" t="s">
+        <x:v>87</x:v>
+      </x:c>
+      <x:c r="D544">
+        <x:v>1010130001</x:v>
+      </x:c>
+      <x:c r="E544">
+        <x:v>-2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="545">
+      <x:c r="A545">
+        <x:v>12.2</x:v>
+      </x:c>
+      <x:c r="B545" t="str">
+        <x:v>DP,DDE st.4.5m</x:v>
+      </x:c>
+      <x:c r="C545" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="D545">
+        <x:v>1010180100</x:v>
+      </x:c>
+      <x:c r="E545">
+        <x:v>12</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="546">
+      <x:c r="A546">
+        <x:v>12.2</x:v>
+      </x:c>
+      <x:c r="B546" t="str">
+        <x:v>DP,DDE st.4.5m</x:v>
+      </x:c>
+      <x:c r="C546" t="s">
+        <x:v>199</x:v>
+      </x:c>
+      <x:c r="D546">
+        <x:v>1010180001</x:v>
+      </x:c>
+      <x:c r="E546">
+        <x:v>6</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="547">
+      <x:c r="A547">
+        <x:v>12.2</x:v>
+      </x:c>
+      <x:c r="B547" t="str">
+        <x:v>DP,DDE st.4.5m</x:v>
+      </x:c>
+      <x:c r="C547" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="D547">
+        <x:v>1010180301</x:v>
+      </x:c>
+      <x:c r="E547">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="548">
+      <x:c r="A548">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="B548" t="str">
+        <x:v>DP,DDE st.4.5m</x:v>
+      </x:c>
+      <x:c r="C548" t="s">
+        <x:v>83</x:v>
+      </x:c>
+      <x:c r="D548" t="s">
+        <x:v>84</x:v>
+      </x:c>
+      <x:c r="E548">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="549">
+      <x:c r="A549">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="B549" t="str">
+        <x:v>DP,DDE st.4.5m</x:v>
+      </x:c>
+      <x:c r="C549" t="s">
+        <x:v>173</x:v>
+      </x:c>
+      <x:c r="D549" t="s">
+        <x:v>174</x:v>
+      </x:c>
+      <x:c r="E549">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="550">
+      <x:c r="A550">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="B550" t="str">
+        <x:v>DP,DDE st.4.5m</x:v>
+      </x:c>
+      <x:c r="C550" t="s">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="D550">
+        <x:v>1010110202</x:v>
+      </x:c>
+      <x:c r="E550">
+        <x:v>4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="551">
+      <x:c r="A551">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="B551" t="str">
+        <x:v>DP,DDE st.4.5m</x:v>
+      </x:c>
+      <x:c r="C551" t="s">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="D551">
+        <x:v>1010110207</x:v>
+      </x:c>
+      <x:c r="E551">
+        <x:v>-1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="552">
+      <x:c r="A552">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="B552" t="str">
+        <x:v>DP,DDE st.4.5m</x:v>
+      </x:c>
+      <x:c r="C552" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="D552">
+        <x:v>1010110209</x:v>
+      </x:c>
+      <x:c r="E552">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="553">
+      <x:c r="A553">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="B553" t="str">
+        <x:v>DP,DDE st.4.5m</x:v>
+      </x:c>
+      <x:c r="C553" t="s">
+        <x:v>87</x:v>
+      </x:c>
+      <x:c r="D553">
+        <x:v>1010130001</x:v>
+      </x:c>
+      <x:c r="E553">
+        <x:v>-2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="554">
+      <x:c r="A554">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="B554" t="str">
+        <x:v>DP,DDE st.4.5m</x:v>
+      </x:c>
+      <x:c r="C554" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="D554">
+        <x:v>1010180100</x:v>
+      </x:c>
+      <x:c r="E554">
+        <x:v>12</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="555">
+      <x:c r="A555">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="B555" t="str">
+        <x:v>DP,DDE st.4.5m</x:v>
+      </x:c>
+      <x:c r="C555" t="s">
+        <x:v>199</x:v>
+      </x:c>
+      <x:c r="D555">
+        <x:v>1010180001</x:v>
+      </x:c>
+      <x:c r="E555">
+        <x:v>6</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="556">
+      <x:c r="A556">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="B556" t="str">
+        <x:v>DP,DDE st.4.5m</x:v>
+      </x:c>
+      <x:c r="C556" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="D556">
+        <x:v>1010180301</x:v>
+      </x:c>
+      <x:c r="E556">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="557">
+      <x:c r="A557">
+        <x:v>14.3</x:v>
+      </x:c>
+      <x:c r="B557" t="str">
+        <x:v>DP,DDE st.4.5m</x:v>
+      </x:c>
+      <x:c r="C557" t="s">
+        <x:v>83</x:v>
+      </x:c>
+      <x:c r="D557" t="s">
+        <x:v>84</x:v>
+      </x:c>
+      <x:c r="E557">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="558">
+      <x:c r="A558">
+        <x:v>14.3</x:v>
+      </x:c>
+      <x:c r="B558" t="str">
+        <x:v>DP,DDE st.4.5m</x:v>
+      </x:c>
+      <x:c r="C558" t="s">
+        <x:v>173</x:v>
+      </x:c>
+      <x:c r="D558" t="s">
+        <x:v>174</x:v>
+      </x:c>
+      <x:c r="E558">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="559">
+      <x:c r="A559">
+        <x:v>14.3</x:v>
+      </x:c>
+      <x:c r="B559" t="str">
+        <x:v>DP,DDE st.4.5m</x:v>
+      </x:c>
+      <x:c r="C559" t="s">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="D559">
+        <x:v>1010110202</x:v>
+      </x:c>
+      <x:c r="E559">
+        <x:v>4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="560">
+      <x:c r="A560">
+        <x:v>14.3</x:v>
+      </x:c>
+      <x:c r="B560" t="str">
+        <x:v>DP,DDE st.4.5m</x:v>
+      </x:c>
+      <x:c r="C560" t="s">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="D560">
+        <x:v>1010110207</x:v>
+      </x:c>
+      <x:c r="E560">
+        <x:v>-1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="561">
+      <x:c r="A561">
+        <x:v>14.3</x:v>
+      </x:c>
+      <x:c r="B561" t="str">
+        <x:v>DP,DDE st.4.5m</x:v>
+      </x:c>
+      <x:c r="C561" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="D561">
+        <x:v>1010110209</x:v>
+      </x:c>
+      <x:c r="E561">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="562">
+      <x:c r="A562">
+        <x:v>14.3</x:v>
+      </x:c>
+      <x:c r="B562" t="str">
+        <x:v>DP,DDE st.4.5m</x:v>
+      </x:c>
+      <x:c r="C562" t="s">
+        <x:v>87</x:v>
+      </x:c>
+      <x:c r="D562">
+        <x:v>1010130001</x:v>
+      </x:c>
+      <x:c r="E562">
+        <x:v>-2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="563">
+      <x:c r="A563">
+        <x:v>14.3</x:v>
+      </x:c>
+      <x:c r="B563" t="str">
+        <x:v>DP,DDE st.4.5m</x:v>
+      </x:c>
+      <x:c r="C563" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="D563">
+        <x:v>1010180100</x:v>
+      </x:c>
+      <x:c r="E563">
+        <x:v>12</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="564">
+      <x:c r="A564">
+        <x:v>14.3</x:v>
+      </x:c>
+      <x:c r="B564" t="str">
+        <x:v>DP,DDE st.4.5m</x:v>
+      </x:c>
+      <x:c r="C564" t="s">
+        <x:v>199</x:v>
+      </x:c>
+      <x:c r="D564">
+        <x:v>1010180001</x:v>
+      </x:c>
+      <x:c r="E564">
+        <x:v>6</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="565">
+      <x:c r="A565">
+        <x:v>14.3</x:v>
+      </x:c>
+      <x:c r="B565" t="str">
+        <x:v>DP,DDE st.4.5m</x:v>
+      </x:c>
+      <x:c r="C565" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="D565">
+        <x:v>1010180301</x:v>
+      </x:c>
+      <x:c r="E565">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8761d97a3a1f47c8"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R32abfb6524f94826"/>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add DP,DE st.4.5m with insulator display counts
</commit_message>
<xml_diff>
--- a/Newdata.xlsx
+++ b/Newdata.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BaseData" sheetId="1" r:id="Rc3d5d22a7d5d4c94"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BaseData" sheetId="1" r:id="R9f0f7496bbdd4aaf"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -11137,8 +11137,433 @@
         <x:v>1</x:v>
       </x:c>
     </x:row>
+    <x:row r="566">
+      <x:c r="A566">
+        <x:v>12.2</x:v>
+      </x:c>
+      <x:c r="B566" t="str">
+        <x:v>DP,DE st.4.5m</x:v>
+      </x:c>
+      <x:c r="C566" t="s">
+        <x:v>83</x:v>
+      </x:c>
+      <x:c r="D566" t="s">
+        <x:v>84</x:v>
+      </x:c>
+      <x:c r="E566">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="567">
+      <x:c r="A567">
+        <x:v>12.2</x:v>
+      </x:c>
+      <x:c r="B567" t="str">
+        <x:v>DP,DE st.4.5m</x:v>
+      </x:c>
+      <x:c r="C567" t="s">
+        <x:v>173</x:v>
+      </x:c>
+      <x:c r="D567" t="s">
+        <x:v>174</x:v>
+      </x:c>
+      <x:c r="E567">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="568">
+      <x:c r="A568">
+        <x:v>12.2</x:v>
+      </x:c>
+      <x:c r="B568" t="str">
+        <x:v>DP,DE st.4.5m</x:v>
+      </x:c>
+      <x:c r="C568" t="s">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="D568">
+        <x:v>1010110202</x:v>
+      </x:c>
+      <x:c r="E568">
+        <x:v>4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="569">
+      <x:c r="A569">
+        <x:v>12.2</x:v>
+      </x:c>
+      <x:c r="B569" t="str">
+        <x:v>DP,DE st.4.5m</x:v>
+      </x:c>
+      <x:c r="C569" t="s">
+        <x:v>87</x:v>
+      </x:c>
+      <x:c r="D569">
+        <x:v>1010130001</x:v>
+      </x:c>
+      <x:c r="E569">
+        <x:v>-2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="570">
+      <x:c r="A570">
+        <x:v>12.2</x:v>
+      </x:c>
+      <x:c r="B570" t="str">
+        <x:v>DP,DE st.4.5m</x:v>
+      </x:c>
+      <x:c r="C570" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="D570">
+        <x:v>1010180100</x:v>
+      </x:c>
+      <x:c r="E570">
+        <x:v>12</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="571">
+      <x:c r="A571">
+        <x:v>12.2</x:v>
+      </x:c>
+      <x:c r="B571" t="str">
+        <x:v>DP,DE st.4.5m</x:v>
+      </x:c>
+      <x:c r="C571" t="s">
+        <x:v>199</x:v>
+      </x:c>
+      <x:c r="D571">
+        <x:v>1010180001</x:v>
+      </x:c>
+      <x:c r="E571">
+        <x:v>6</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="572">
+      <x:c r="A572">
+        <x:v>12.2</x:v>
+      </x:c>
+      <x:c r="B572" t="str">
+        <x:v>DP,DE st.4.5m</x:v>
+      </x:c>
+      <x:c r="C572" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="D572">
+        <x:v>1010180301</x:v>
+      </x:c>
+      <x:c r="E572">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="573">
+      <x:c r="A573">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="B573" t="str">
+        <x:v>DP,DE st.4.5m</x:v>
+      </x:c>
+      <x:c r="C573" t="s">
+        <x:v>83</x:v>
+      </x:c>
+      <x:c r="D573" t="s">
+        <x:v>84</x:v>
+      </x:c>
+      <x:c r="E573">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="574">
+      <x:c r="A574">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="B574" t="str">
+        <x:v>DP,DE st.4.5m</x:v>
+      </x:c>
+      <x:c r="C574" t="s">
+        <x:v>173</x:v>
+      </x:c>
+      <x:c r="D574" t="s">
+        <x:v>174</x:v>
+      </x:c>
+      <x:c r="E574">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="575">
+      <x:c r="A575">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="B575" t="str">
+        <x:v>DP,DE st.4.5m</x:v>
+      </x:c>
+      <x:c r="C575" t="s">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="D575">
+        <x:v>1010110202</x:v>
+      </x:c>
+      <x:c r="E575">
+        <x:v>4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="576">
+      <x:c r="A576">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="B576" t="str">
+        <x:v>DP,DE st.4.5m</x:v>
+      </x:c>
+      <x:c r="C576" t="s">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="D576">
+        <x:v>1010110207</x:v>
+      </x:c>
+      <x:c r="E576">
+        <x:v>-1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="577">
+      <x:c r="A577">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="B577" t="str">
+        <x:v>DP,DE st.4.5m</x:v>
+      </x:c>
+      <x:c r="C577" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="D577">
+        <x:v>1010110209</x:v>
+      </x:c>
+      <x:c r="E577">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="578">
+      <x:c r="A578">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="B578" t="str">
+        <x:v>DP,DE st.4.5m</x:v>
+      </x:c>
+      <x:c r="C578" t="s">
+        <x:v>87</x:v>
+      </x:c>
+      <x:c r="D578">
+        <x:v>1010130001</x:v>
+      </x:c>
+      <x:c r="E578">
+        <x:v>-2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="579">
+      <x:c r="A579">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="B579" t="str">
+        <x:v>DP,DE st.4.5m</x:v>
+      </x:c>
+      <x:c r="C579" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="D579">
+        <x:v>1010180100</x:v>
+      </x:c>
+      <x:c r="E579">
+        <x:v>12</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="580">
+      <x:c r="A580">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="B580" t="str">
+        <x:v>DP,DE st.4.5m</x:v>
+      </x:c>
+      <x:c r="C580" t="s">
+        <x:v>199</x:v>
+      </x:c>
+      <x:c r="D580">
+        <x:v>1010180001</x:v>
+      </x:c>
+      <x:c r="E580">
+        <x:v>6</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="581">
+      <x:c r="A581">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="B581" t="str">
+        <x:v>DP,DE st.4.5m</x:v>
+      </x:c>
+      <x:c r="C581" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="D581">
+        <x:v>1010180301</x:v>
+      </x:c>
+      <x:c r="E581">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="582">
+      <x:c r="A582">
+        <x:v>14.3</x:v>
+      </x:c>
+      <x:c r="B582" t="str">
+        <x:v>DP,DE st.4.5m</x:v>
+      </x:c>
+      <x:c r="C582" t="s">
+        <x:v>83</x:v>
+      </x:c>
+      <x:c r="D582" t="s">
+        <x:v>84</x:v>
+      </x:c>
+      <x:c r="E582">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="583">
+      <x:c r="A583">
+        <x:v>14.3</x:v>
+      </x:c>
+      <x:c r="B583" t="str">
+        <x:v>DP,DE st.4.5m</x:v>
+      </x:c>
+      <x:c r="C583" t="s">
+        <x:v>173</x:v>
+      </x:c>
+      <x:c r="D583" t="s">
+        <x:v>174</x:v>
+      </x:c>
+      <x:c r="E583">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="584">
+      <x:c r="A584">
+        <x:v>14.3</x:v>
+      </x:c>
+      <x:c r="B584" t="str">
+        <x:v>DP,DE st.4.5m</x:v>
+      </x:c>
+      <x:c r="C584" t="s">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="D584">
+        <x:v>1010110202</x:v>
+      </x:c>
+      <x:c r="E584">
+        <x:v>4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="585">
+      <x:c r="A585">
+        <x:v>14.3</x:v>
+      </x:c>
+      <x:c r="B585" t="str">
+        <x:v>DP,DE st.4.5m</x:v>
+      </x:c>
+      <x:c r="C585" t="s">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="D585">
+        <x:v>1010110207</x:v>
+      </x:c>
+      <x:c r="E585">
+        <x:v>-1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="586">
+      <x:c r="A586">
+        <x:v>14.3</x:v>
+      </x:c>
+      <x:c r="B586" t="str">
+        <x:v>DP,DE st.4.5m</x:v>
+      </x:c>
+      <x:c r="C586" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="D586">
+        <x:v>1010110209</x:v>
+      </x:c>
+      <x:c r="E586">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="587">
+      <x:c r="A587">
+        <x:v>14.3</x:v>
+      </x:c>
+      <x:c r="B587" t="str">
+        <x:v>DP,DE st.4.5m</x:v>
+      </x:c>
+      <x:c r="C587" t="s">
+        <x:v>87</x:v>
+      </x:c>
+      <x:c r="D587">
+        <x:v>1010130001</x:v>
+      </x:c>
+      <x:c r="E587">
+        <x:v>-2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="588">
+      <x:c r="A588">
+        <x:v>14.3</x:v>
+      </x:c>
+      <x:c r="B588" t="str">
+        <x:v>DP,DE st.4.5m</x:v>
+      </x:c>
+      <x:c r="C588" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="D588">
+        <x:v>1010180100</x:v>
+      </x:c>
+      <x:c r="E588">
+        <x:v>12</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="589">
+      <x:c r="A589">
+        <x:v>14.3</x:v>
+      </x:c>
+      <x:c r="B589" t="str">
+        <x:v>DP,DE st.4.5m</x:v>
+      </x:c>
+      <x:c r="C589" t="s">
+        <x:v>199</x:v>
+      </x:c>
+      <x:c r="D589">
+        <x:v>1010180001</x:v>
+      </x:c>
+      <x:c r="E589">
+        <x:v>6</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="590">
+      <x:c r="A590">
+        <x:v>14.3</x:v>
+      </x:c>
+      <x:c r="B590" t="str">
+        <x:v>DP,DE st.4.5m</x:v>
+      </x:c>
+      <x:c r="C590" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="D590">
+        <x:v>1010180301</x:v>
+      </x:c>
+      <x:c r="E590">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R32abfb6524f94826"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5946adc754884b4e"/>
 </x:worksheet>
 </file>
</xml_diff>